<commit_message>
feat(dashboard): adicionar tabela consolidada com 1 stop red por metodo na pagina 02 e relatorios de auditoria
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-24.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-24.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,26 +509,6 @@
           <t>Liquidez_Lay</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Hora_Str</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Risco_Red_R$</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Stake_Sugerida_R$</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Lucro_Green_R$</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -543,27 +523,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Vietnamese V-League</t>
+          <t>German Bundesliga 2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Truong Tuoi Dong Nai x Nam Dinh</t>
+          <t>FC Heidenheim x Cottbus</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Truong Tuoi Dong Nai</t>
+          <t>FC Heidenheim</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Nam Dinh</t>
+          <t>Cottbus</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -573,14 +553,14 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>6.2</v>
+        <v>16</v>
       </c>
       <c r="K2" t="n">
-        <v>1.62</v>
+        <v>1.53</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>AO Away Win</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -599,21 +579,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>225</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
-        <v>200</v>
-      </c>
-      <c r="S2" t="n">
-        <v>38.46</v>
-      </c>
-      <c r="T2" t="n">
-        <v>36.73</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3">
@@ -624,32 +590,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>English Sky Bet League 1</t>
+          <t>Vietnamese V-League</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Huddersfield x Wigan</t>
+          <t>Truong Tuoi Dong Nai x Nam Dinh</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Huddersfield</t>
+          <t>Truong Tuoi Dong Nai</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Wigan</t>
+          <t>Nam Dinh</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -659,14 +625,14 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="K3" t="n">
-        <v>1.38</v>
+        <v>1.62</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>AO Away Win</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -685,21 +651,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>1095</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>200</v>
-      </c>
-      <c r="S3" t="n">
-        <v>41.67</v>
-      </c>
-      <c r="T3" t="n">
-        <v>39.79</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4">
@@ -715,27 +667,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Danish 1st Division</t>
+          <t>English Sky Bet League 1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Esbjerg x Fredericia</t>
+          <t>Huddersfield x Wigan</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Esbjerg</t>
+          <t>Huddersfield</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Fredericia</t>
+          <t>Wigan</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -748,7 +700,7 @@
         <v>5.8</v>
       </c>
       <c r="K4" t="n">
-        <v>1.58</v>
+        <v>1.38</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -757,7 +709,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -771,21 +723,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>760</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>200</v>
-      </c>
-      <c r="S4" t="n">
-        <v>41.67</v>
-      </c>
-      <c r="T4" t="n">
-        <v>39.79</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="5">
@@ -796,32 +734,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Swedish Allsvenskan</t>
+          <t>Danish 1st Division</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hacken x Degerfors</t>
+          <t>Esbjerg x Fredericia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Hacken</t>
+          <t>Esbjerg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Degerfors</t>
+          <t>Fredericia</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -831,19 +769,19 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="K5" t="n">
-        <v>1.39</v>
+        <v>1.58</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>AO Home Win</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -857,21 +795,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>1361</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>200</v>
-      </c>
-      <c r="S5" t="n">
-        <v>40.82</v>
-      </c>
-      <c r="T5" t="n">
-        <v>38.98</v>
+        <v>760</v>
       </c>
     </row>
     <row r="6">
@@ -882,27 +806,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>English Premier League</t>
+          <t>Swedish Allsvenskan</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Arsenal x Everton</t>
+          <t>Hacken x Degerfors</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>Hacken</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Everton</t>
+          <t>Degerfors</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -917,14 +841,14 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="K6" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>AO Home Win</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -943,21 +867,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>11036</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
-        <v>200</v>
-      </c>
-      <c r="S6" t="n">
-        <v>43.48</v>
-      </c>
-      <c r="T6" t="n">
-        <v>41.52</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="7">
@@ -973,22 +883,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>English National League</t>
+          <t>English Premier League</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Boreham Wood x AFC Fylde</t>
+          <t>Arsenal x Everton</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Boreham Wood</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AFC Fylde</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1003,14 +913,14 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
       <c r="K7" t="n">
-        <v>1.4</v>
+        <v>1.38</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>AO Home Win</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1029,21 +939,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>469</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R7" t="n">
-        <v>200</v>
-      </c>
-      <c r="S7" t="n">
-        <v>37.04</v>
-      </c>
-      <c r="T7" t="n">
-        <v>35.37</v>
+        <v>11036</v>
       </c>
     </row>
     <row r="8">
@@ -1059,22 +955,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Scottish League One</t>
+          <t>English National League</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ross Co x Airdrieonians</t>
+          <t>Boreham Wood x AFC Fylde</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ross Co</t>
+          <t>Boreham Wood</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Airdrieonians</t>
+          <t>AFC Fylde</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1089,10 +985,10 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="K8" t="n">
-        <v>1.32</v>
+        <v>1.4</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -1115,21 +1011,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>269</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R8" t="n">
-        <v>200</v>
-      </c>
-      <c r="S8" t="n">
-        <v>35.71</v>
-      </c>
-      <c r="T8" t="n">
-        <v>34.1</v>
+        <v>469</v>
       </c>
     </row>
     <row r="9">
@@ -1145,27 +1027,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Scottish Championship</t>
+          <t>Scottish League One</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Queens Park x Dunfermline</t>
+          <t>Ross Co x Airdrieonians</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Queens Park</t>
+          <t>Ross Co</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Dunfermline</t>
+          <t>Airdrieonians</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1175,14 +1057,14 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="K9" t="n">
-        <v>1.6</v>
+        <v>1.32</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>AO Home Win</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1201,21 +1083,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>766</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="R9" t="n">
-        <v>200</v>
-      </c>
-      <c r="S9" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="T9" t="n">
-        <v>31.83</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10">
@@ -1226,32 +1094,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ukrainian Premier League</t>
+          <t>Scottish Championship</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Shakhtar x Zorya</t>
+          <t>Queens Park x Dunfermline</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Shakhtar</t>
+          <t>Queens Park</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Zorya</t>
+          <t>Dunfermline</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1261,19 +1129,19 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>5.6</v>
+        <v>7</v>
       </c>
       <c r="K10" t="n">
-        <v>1.36</v>
+        <v>1.6</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1287,21 +1155,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>640</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="R10" t="n">
-        <v>200</v>
-      </c>
-      <c r="S10" t="n">
-        <v>43.48</v>
-      </c>
-      <c r="T10" t="n">
-        <v>41.52</v>
+        <v>766</v>
       </c>
     </row>
     <row r="11">
@@ -1312,32 +1166,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Norwegian Eliteserien</t>
+          <t>Ukrainian Premier League</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ham-Kam x Rosenborg</t>
+          <t>Shakhtar x Zorya</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ham-Kam</t>
+          <t>Shakhtar</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Rosenborg</t>
+          <t>Zorya</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1347,19 +1201,19 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>6.2</v>
+        <v>5.6</v>
       </c>
       <c r="K11" t="n">
-        <v>1.58</v>
+        <v>1.36</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1373,21 +1227,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>2358</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="R11" t="n">
-        <v>200</v>
-      </c>
-      <c r="S11" t="n">
-        <v>38.46</v>
-      </c>
-      <c r="T11" t="n">
-        <v>36.73</v>
+        <v>640</v>
       </c>
     </row>
     <row r="12">
@@ -1398,32 +1238,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Spanish Segunda Division</t>
+          <t>Norwegian Eliteserien</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Girona x Celta Vigo B</t>
+          <t>Ham-Kam x Rosenborg</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Ham-Kam</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Celta Vigo B</t>
+          <t>Rosenborg</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1433,14 +1273,14 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>5.6</v>
+        <v>6.2</v>
       </c>
       <c r="K12" t="n">
-        <v>1.4</v>
+        <v>1.58</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>AO Home Win</t>
+          <t>0-3</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1459,21 +1299,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>1714</v>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="R12" t="n">
-        <v>200</v>
-      </c>
-      <c r="S12" t="n">
-        <v>43.48</v>
-      </c>
-      <c r="T12" t="n">
-        <v>41.52</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="13">
@@ -1484,32 +1310,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>US MLS</t>
+          <t>Spanish Segunda Division</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CF Montreal x Nashville SC</t>
+          <t>Girona x Celta Vigo B</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CF Montreal</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Nashville SC</t>
+          <t>Celta Vigo B</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1519,14 +1345,14 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>7.8</v>
+        <v>5.6</v>
       </c>
       <c r="K13" t="n">
-        <v>1.49</v>
+        <v>1.4</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>AO Home Win</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1545,21 +1371,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>4273</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="R13" t="n">
-        <v>200</v>
-      </c>
-      <c r="S13" t="n">
-        <v>29.41</v>
-      </c>
-      <c r="T13" t="n">
-        <v>28.09</v>
+        <v>1714</v>
       </c>
     </row>
     <row r="14">
@@ -1570,32 +1382,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Colombian Primera B</t>
+          <t>US MLS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Union Magdalena x Atletico FC Cali</t>
+          <t>CF Montreal x Nashville SC</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Union Magdalena</t>
+          <t>CF Montreal</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Atletico FC Cali</t>
+          <t>Nashville SC</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1605,14 +1417,14 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="K14" t="n">
-        <v>1.3</v>
+        <v>1.49</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1631,21 +1443,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>1260</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="R14" t="n">
-        <v>200</v>
-      </c>
-      <c r="S14" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="T14" t="n">
-        <v>31.83</v>
+        <v>4273</v>
       </c>
     </row>
     <row r="15">
@@ -1656,27 +1454,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Brazilian Serie B</t>
+          <t>Colombian Primera B</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CRB x Londrina</t>
+          <t>Union Magdalena x Atletico FC Cali</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Union Magdalena</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Atletico FC Cali</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1691,14 +1489,14 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="K15" t="n">
-        <v>1.36</v>
+        <v>1.3</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1717,21 +1515,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>1274</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="R15" t="n">
-        <v>200</v>
-      </c>
-      <c r="S15" t="n">
-        <v>38.46</v>
-      </c>
-      <c r="T15" t="n">
-        <v>36.73</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="16">
@@ -1752,17 +1536,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ponte Preta x Fortaleza EC</t>
+          <t>CRB x Londrina</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Fortaleza EC</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1777,47 +1561,105 @@
         </is>
       </c>
       <c r="J16" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Brazilian Serie B</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ponte Preta x Fortaleza EC</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Fortaleza EC</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
         <v>6.8</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K17" t="n">
         <v>1.26</v>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>2-2</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>RED</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>✅ LIQUIDADO</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>coletor (KO-10)</t>
         </is>
       </c>
-      <c r="P16" t="n">
+      <c r="P17" t="n">
         <v>283</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="R16" t="n">
-        <v>200</v>
-      </c>
-      <c r="S16" t="n">
-        <v>34.48</v>
-      </c>
-      <c r="T16" t="n">
-        <v>32.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>